<commit_message>
sync: 2 file(s) changed — 2026-08-23 23:18
</commit_message>
<xml_diff>
--- a/outputs/inc42/Inc42 Web Analytics — Event Register.xlsx
+++ b/outputs/inc42/Inc42 Web Analytics — Event Register.xlsx
@@ -15,10 +15,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scroll Depth" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Re-Audit vs June'!$A$4:$I$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Re-Audit vs June'!$A$4:$I$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Event Register'!$A$4:$L$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Property Dictionary'!$A$4:$H$118</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Findings'!$A$4:$G$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Findings'!$A$4:$G$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -871,7 +871,7 @@
         <is>
           <t>Spec: 'Inc42 Website - Events &amp; Properties.xlsx' (v1.0, 12 Aug 2026).
 Warehouse: 'Inc42 Analytics | Master.xlsx' tab 'Audit | Jun 2026' (PostHog 53557, 30d to 22 Jun 2026).
-Browser: automated audit, run 2026-08-23 17:26.</t>
+Browser: automated audit, run 2026-08-23 17:39.</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Every event from the Master sheet's latest tab, re-tested in a live browser on 2026-08-23 17:26. 'not tested' rows are honest gaps, not defects — the trigger never occurred or the journey needs credentials.</t>
+          <t>Every event from the Master sheet's latest tab, re-tested in a live browser on 2026-08-23 17:39. 'not tested' rows are honest gaps, not defects — the trigger never occurred or the journey needs credentials.</t>
         </is>
       </c>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>ga4 ×26</t>
+          <t>ga4 ×35</t>
         </is>
       </c>
       <c r="G5" s="11" t="inlineStr">
@@ -1078,7 +1078,7 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Ad Blocker</t>
+          <t>App Banner Viewed</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -1095,7 +1095,7 @@
       <c r="E7" s="9" t="inlineStr"/>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>ga4 ×3</t>
+          <t>ga4 ×45</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Ad Blocker is live but absent from the June audit</t>
+          <t>App Banner Viewed is live but absent from the June audit</t>
         </is>
       </c>
       <c r="I7" s="13" t="inlineStr">
@@ -1117,34 +1117,40 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>App Banner Viewed</t>
+          <t>My Inc42</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>absent</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="n"/>
+          <t>⚠️ Dead</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n">
+        <v>1</v>
+      </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>— none reaches it</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr"/>
+          <t>logged-in</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>personalised feed opened</t>
+        </is>
+      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
-          <t>ga4 ×28</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>App Banner Viewed is live but absent from the June audit</t>
+          <t>My Inc42 is still not firing</t>
         </is>
       </c>
       <c r="I8" s="13" t="inlineStr">
@@ -1156,40 +1162,34 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Search Click</t>
+          <t>Scroll Depth</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>🔵 Name drift</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>531</v>
-      </c>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n"/>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>search</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>search result opened</t>
-        </is>
-      </c>
+          <t>— none reaches it</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>nothing</t>
+          <t>ga4 ×2</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>unchanged</t>
+          <t>new</t>
         </is>
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Search Click is still not firing</t>
+          <t>Scroll Depth is live but absent from the June audit</t>
         </is>
       </c>
       <c r="I9" s="13" t="inlineStr">
@@ -1201,25 +1201,25 @@
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Share</t>
+          <t>Search Click</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>✅ Healthy</t>
+          <t>🔵 Name drift</t>
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>32</v>
+        <v>531</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>share</t>
+          <t>search</t>
         </is>
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>share action on an article</t>
+          <t>search result opened</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -1234,7 +1234,7 @@
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Share is still not firing</t>
+          <t>Search Click is still not firing</t>
         </is>
       </c>
       <c r="I10" s="13" t="inlineStr">
@@ -1246,34 +1246,40 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>scroll</t>
+          <t>Share</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>absent</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="n"/>
+          <t>✅ Healthy</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>32</v>
+      </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>— none reaches it</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr"/>
+          <t>share</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>share action on an article</t>
+        </is>
+      </c>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>ga4 ×16</t>
+          <t>nothing</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>unchanged</t>
         </is>
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>scroll is live but absent from the June audit</t>
+          <t>Share is still not firing</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
@@ -1285,70 +1291,64 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Follow</t>
+          <t>scroll</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>⚠️ Near-zero</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="n">
-        <v>4</v>
-      </c>
+          <t>absent</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="n"/>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>logged-in</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>follow an entity</t>
-        </is>
-      </c>
+          <t>— none reaches it</t>
+        </is>
+      </c>
+      <c r="E12" s="9" t="inlineStr"/>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>nothing</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>not tested</t>
+          <t>ga4 ×18</t>
+        </is>
+      </c>
+      <c r="G12" s="13" t="inlineStr">
+        <is>
+          <t>new</t>
         </is>
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Follow — its journey did not run</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>scroll is live but absent from the June audit</t>
+        </is>
+      </c>
+      <c r="I12" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Freewall Lock</t>
+          <t>Follow</t>
         </is>
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>✅ Healthy</t>
+          <t>⚠️ Near-zero</t>
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>59561</v>
+        <v>4</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
-          <t>freewall</t>
+          <t>logged-in</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>register gate renders</t>
+          <t>follow an entity</t>
         </is>
       </c>
       <c r="F13" s="8" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>Freewall Lock — the trigger never occurred</t>
+          <t>Follow — the trigger never occurred</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
@@ -1375,7 +1375,7 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Login</t>
+          <t>Freewall Lock</t>
         </is>
       </c>
       <c r="B14" s="9" t="inlineStr">
@@ -1384,16 +1384,16 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>3136</v>
+        <v>59561</v>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>logged-in</t>
+          <t>freewall</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>auth succeeds</t>
+          <t>register gate renders</t>
         </is>
       </c>
       <c r="F14" s="8" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>Login — its journey did not run</t>
+          <t>Freewall Lock — the trigger never occurred</t>
         </is>
       </c>
       <c r="I14" s="14" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>logged-in</t>
+          <t>logout</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
@@ -1498,7 +1498,7 @@
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>Logout — its journey did not run</t>
+          <t>Logout — the trigger never occurred</t>
         </is>
       </c>
       <c r="I16" s="14" t="inlineStr">
@@ -1690,25 +1690,25 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>My Inc42</t>
+          <t>Qr Scan</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>⚠️ Dead</t>
+          <t>⚠️ Near-zero</t>
         </is>
       </c>
       <c r="C21" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>logged-in</t>
+          <t>— none reaches it</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>personalised feed opened</t>
+          <t>QR landing</t>
         </is>
       </c>
       <c r="F21" s="8" t="inlineStr">
@@ -1718,12 +1718,12 @@
       </c>
       <c r="G21" s="14" t="inlineStr">
         <is>
-          <t>not tested</t>
+          <t>unchanged, unverified</t>
         </is>
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>My Inc42 — its journey did not run</t>
+          <t>Qr Scan — June flagged it, no journey can reach it</t>
         </is>
       </c>
       <c r="I21" s="14" t="inlineStr">
@@ -1735,7 +1735,7 @@
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Qr Scan</t>
+          <t>Save Story</t>
         </is>
       </c>
       <c r="B22" s="9" t="inlineStr">
@@ -1744,31 +1744,31 @@
         </is>
       </c>
       <c r="C22" s="10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>— none reaches it</t>
+          <t>logged-in</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>QR landing</t>
+          <t>bookmark an article</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
-          <t>nothing</t>
-        </is>
-      </c>
-      <c r="G22" s="14" t="inlineStr">
-        <is>
-          <t>unchanged, unverified</t>
+          <t>posthog ×1, ga4 ×1</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>improved since June</t>
         </is>
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>Qr Scan — June flagged it, no journey can reach it</t>
+          <t>Save Story is firing again</t>
         </is>
       </c>
       <c r="I22" s="14" t="inlineStr">
@@ -1780,25 +1780,25 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Save Story</t>
+          <t>Unfollow</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>⚠️ Near-zero</t>
+          <t>⚠️ Dead</t>
         </is>
       </c>
       <c r="C23" s="10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>logged-in</t>
+          <t>— none reaches it</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>bookmark an article</t>
+          <t>unfollow</t>
         </is>
       </c>
       <c r="F23" s="8" t="inlineStr">
@@ -1808,12 +1808,12 @@
       </c>
       <c r="G23" s="14" t="inlineStr">
         <is>
-          <t>not tested</t>
+          <t>unchanged, unverified</t>
         </is>
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>Save Story — its journey did not run</t>
+          <t>Unfollow — June flagged it, no journey can reach it</t>
         </is>
       </c>
       <c r="I23" s="14" t="inlineStr">
@@ -1825,7 +1825,7 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Unfollow</t>
+          <t>User Segment</t>
         </is>
       </c>
       <c r="B24" s="9" t="inlineStr">
@@ -1838,12 +1838,12 @@
       </c>
       <c r="D24" s="9" t="inlineStr">
         <is>
-          <t>logged-in</t>
+          <t>— none reaches it</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>unfollow</t>
+          <t>MoEngage segment sync</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1853,12 +1853,12 @@
       </c>
       <c r="G24" s="14" t="inlineStr">
         <is>
-          <t>not tested</t>
+          <t>unchanged, unverified</t>
         </is>
       </c>
       <c r="H24" s="12" t="inlineStr">
         <is>
-          <t>Unfollow — its journey did not run</t>
+          <t>User Segment — June flagged it, no journey can reach it</t>
         </is>
       </c>
       <c r="I24" s="14" t="inlineStr">
@@ -1867,62 +1867,58 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="8" t="inlineStr">
-        <is>
-          <t>User Segment</t>
-        </is>
-      </c>
-      <c r="B25" s="9" t="inlineStr">
-        <is>
-          <t>⚠️ Dead</t>
-        </is>
-      </c>
-      <c r="C25" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="9" t="inlineStr">
-        <is>
-          <t>— none reaches it</t>
-        </is>
-      </c>
-      <c r="E25" s="9" t="inlineStr">
-        <is>
-          <t>MoEngage segment sync</t>
-        </is>
-      </c>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>nothing</t>
-        </is>
-      </c>
-      <c r="G25" s="14" t="inlineStr">
-        <is>
-          <t>unchanged, unverified</t>
-        </is>
-      </c>
-      <c r="H25" s="12" t="inlineStr">
-        <is>
-          <t>User Segment — June flagged it, no journey can reach it</t>
-        </is>
-      </c>
-      <c r="I25" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>EVENTS THAT NEEDED NO FLAG</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>EVENTS THAT NEEDED NO FLAG</t>
-        </is>
-      </c>
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>$pageview</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>✅ Healthy</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="n">
+        <v>624466</v>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>article-read</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>any page load</t>
+        </is>
+      </c>
+      <c r="F27" s="8" t="inlineStr">
+        <is>
+          <t>posthog ×31</t>
+        </is>
+      </c>
+      <c r="G27" s="15" t="inlineStr">
+        <is>
+          <t>confirmed firing</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Observed reaching PostHog this run.</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>$pageview</t>
+          <t>Private Mode Modal</t>
         </is>
       </c>
       <c r="B28" s="9" t="inlineStr">
@@ -1931,7 +1927,7 @@
         </is>
       </c>
       <c r="C28" s="10" t="n">
-        <v>624466</v>
+        <v>152639</v>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
@@ -1940,12 +1936,12 @@
       </c>
       <c r="E28" s="9" t="inlineStr">
         <is>
-          <t>any page load</t>
+          <t>modal on load</t>
         </is>
       </c>
       <c r="F28" s="8" t="inlineStr">
         <is>
-          <t>posthog ×21</t>
+          <t>posthog ×36</t>
         </is>
       </c>
       <c r="G28" s="15" t="inlineStr">
@@ -1963,7 +1959,7 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Private Mode Modal</t>
+          <t>Search Completed</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1972,21 +1968,21 @@
         </is>
       </c>
       <c r="C29" s="10" t="n">
-        <v>152639</v>
+        <v>8522</v>
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>article-read</t>
+          <t>search</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
         <is>
-          <t>modal on load</t>
+          <t>query submitted</t>
         </is>
       </c>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>posthog ×26</t>
+          <t>posthog ×1</t>
         </is>
       </c>
       <c r="G29" s="15" t="inlineStr">
@@ -2004,62 +2000,50 @@
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Search Completed</t>
+          <t>Form Submission</t>
         </is>
       </c>
       <c r="B30" s="9" t="inlineStr">
         <is>
-          <t>✅ Healthy</t>
+          <t>🐞 Healthy + bug</t>
         </is>
       </c>
       <c r="C30" s="10" t="n">
-        <v>8522</v>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>search</t>
-        </is>
-      </c>
+        <v>5337</v>
+      </c>
+      <c r="D30" s="9" t="inlineStr"/>
       <c r="E30" s="9" t="inlineStr">
         <is>
-          <t>query submitted</t>
+          <t>any site form</t>
         </is>
       </c>
       <c r="F30" s="8" t="inlineStr">
         <is>
-          <t>posthog ×1</t>
-        </is>
-      </c>
-      <c r="G30" s="15" t="inlineStr">
-        <is>
-          <t>confirmed firing</t>
-        </is>
-      </c>
-      <c r="H30" s="9" t="inlineStr">
-        <is>
-          <t>Observed reaching PostHog this run.</t>
-        </is>
-      </c>
+          <t>nothing</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr"/>
+      <c r="H30" s="9" t="inlineStr"/>
       <c r="I30" s="9" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>Form Submission</t>
+          <t>Login</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
         <is>
-          <t>🐞 Healthy + bug</t>
+          <t>✅ Healthy</t>
         </is>
       </c>
       <c r="C31" s="10" t="n">
-        <v>5337</v>
+        <v>3136</v>
       </c>
       <c r="D31" s="9" t="inlineStr"/>
       <c r="E31" s="9" t="inlineStr">
         <is>
-          <t>any site form</t>
+          <t>auth succeeds</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -2374,7 +2358,7 @@
       <c r="I41" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:I25"/>
+  <autoFilter ref="A4:I24"/>
   <mergeCells count="2">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
@@ -3056,7 +3040,11 @@
       <c r="F16" s="10" t="n">
         <v>7</v>
       </c>
-      <c r="G16" s="12" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
       <c r="H16" s="9" t="inlineStr">
         <is>
           <t>PostHog·Customer.io</t>
@@ -9390,7 +9378,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -9412,7 +9400,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Automated audit, run 2026-08-23 17:26. Browser half only unless a PostHog key was supplied — 'Unverified' rows resolve once the warehouse query runs.</t>
+          <t>Automated audit, run 2026-08-23 17:39. Browser half only unless a PostHog key was supplied — 'Unverified' rows resolve once the warehouse query runs.</t>
         </is>
       </c>
     </row>
@@ -9461,32 +9449,32 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>NOT_INSTRUMENTED</t>
+          <t>NEVER_IDENTIFIED</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>newsletter_prompt_shown</t>
+          <t>(identity)</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
-          <t>newsletter_prompt_shown is not instrumented at all</t>
+          <t>Logged in to the site, anonymous in PostHog</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>No production event is mapped to this spec event (status: partial).</t>
+          <t>Across 8 snapshots in an authenticated session, every distinct_id was an anonymous UUID (e.g. 01a02fb4-02ac-7429-9080-e47bfd8223b4). Never an email, never an Auth0 id. identify() did not fire.</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Prompt→subscribe funnel denominator</t>
+          <t>Logged-in behaviour cannot be attributed to a person. Every funnel that joins anonymous reading to a known user breaks here, and this is the mechanism behind the low web identification rate.</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Instrument newsletter_prompt_shown per the spec — fires when: A subscribe prompt is displayed (inline / footer / exit-popup).</t>
+          <t>Call posthog.identify() with the Auth0 uid on every page load for an authenticated user, not only at the moment of login. Keep email as a $set property.</t>
         </is>
       </c>
     </row>
@@ -9498,32 +9486,32 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>VENDOR_BALANCE</t>
+          <t>NEVER_IDENTIFIED</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>(stack)</t>
+          <t>(identity)</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
         <is>
-          <t>GA4 receives 9 distinct events; PostHog receives 6</t>
+          <t>Customer.io holds a guest token for a signed-in user</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
         <is>
-          <t>Across every journey in this run: ga4 9 · posthog 6 · customerio 1.</t>
+          <t>analytics.user().id() was null in all 8 authenticated snapshots. The saved session also carries a gist.web.usingGuestUserToken key in localStorage.</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>Product analytics is the thinner dataset. Every product decision is made on the tool with less information.</t>
+          <t>Every browser-side Customer.io event is attributed to a guest. Lifecycle messaging depends entirely on server-side/reverse-ETL, with no real-time site behaviour and no client-side fallback.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
-          <t>Treat the PostHog payload as the contract and mirror to marketing tools, not the other way round.</t>
+          <t>Call the Customer.io identify() on auth, and document client vs server event ownership.</t>
         </is>
       </c>
     </row>
@@ -9535,217 +9523,217 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
+          <t>NOT_INSTRUMENTED</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>newsletter_prompt_shown</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>newsletter_prompt_shown is not instrumented at all</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>No production event is mapped to this spec event (status: partial).</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>Prompt→subscribe funnel denominator</t>
+        </is>
+      </c>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>Instrument newsletter_prompt_shown per the spec — fires when: A subscribe prompt is displayed (inline / footer / exit-popup).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>PII_LEAK</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>(privacy)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Raw email in dataLayer</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Found at dataLayer.0.email (sample "ranjit…") on /.</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>Exposed to every GTM tag and shipped to third parties. Direct DPDP exposure (May-2027).</t>
+        </is>
+      </c>
+      <c r="G8" s="9" t="inlineStr">
+        <is>
+          <t>Send hashed identifiers only client-side; strip raw email/phone from the dataLayer and the shared analytics bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>PII_LEAK</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>(privacy)</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Raw email in eventProperties</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Found at eventProperties.email (sample "ranjit…") on /.</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>Exposed to every GTM tag and shipped to third parties. Direct DPDP exposure (May-2027).</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>Send hashed identifiers only client-side; strip raw email/phone from the dataLayer and the shared analytics bundle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>PII_LEAK</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>(privacy)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Identifiers sent to gtm, ga4</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>127 outbound payload(s) carried email-shaped or ud[]/em/ph/fn/ln fields.</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>Third-party sharing of personal data; needs a consent basis under DPDP.</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>Confirm the consent basis, or disable advanced matching / CAPI PII.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
           <t>VENDOR_BALANCE</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C11" s="8" t="inlineStr">
         <is>
           <t>(stack)</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>GA4 receives 10 distinct events; PostHog receives 8</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
+          <t>Across every journey in this run: ga4 10 · customerio 1 · posthog 8.</t>
+        </is>
+      </c>
+      <c r="F11" s="9" t="inlineStr">
+        <is>
+          <t>Product analytics is the thinner dataset. Every product decision is made on the tool with less information.</t>
+        </is>
+      </c>
+      <c r="G11" s="9" t="inlineStr">
+        <is>
+          <t>Treat the PostHog payload as the contract and mirror to marketing tools, not the other way round.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="inlineStr">
+        <is>
+          <t>VENDOR_BALANCE</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>(stack)</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
         <is>
           <t>Customer.io receives page calls but zero track calls</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>20 outbound Customer.io calls this run, all of type "page". No track() at all.</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>28 outbound Customer.io calls this run, all of type "page". No track() at all.</t>
+        </is>
+      </c>
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>All lifecycle messaging depends on server-side/reverse-ETL. No real-time site behaviour reaches the CRM, and the browser path is a silent single point of failure.</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G12" s="9" t="inlineStr">
         <is>
           <t>Decide client vs server event ownership explicitly and document it; wire track() for the behaviours campaigns trigger on.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>App Banner Viewed</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>App Banner Viewed reaches ga4 but never PostHog</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>28 captures to ga4 during this run; 0 to PostHog.</t>
-        </is>
-      </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
-        </is>
-      </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="13" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Plus Lock</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>Plus Lock reaches ga4 but never PostHog</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
-        <is>
-          <t>26 captures to ga4 during this run; 0 to PostHog.</t>
-        </is>
-      </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
-        </is>
-      </c>
-      <c r="G9" s="9" t="inlineStr">
-        <is>
-          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="13" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="C10" s="8" t="inlineStr">
-        <is>
-          <t>scroll</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>scroll reaches ga4 but never PostHog</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>16 captures to ga4 during this run; 0 to PostHog.</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>COVERAGE_GAP</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Ad Blocker</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>Ad Blocker reaches ga4 but never PostHog</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>3 captures to ga4 during this run; 0 to PostHog.</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
-        </is>
-      </c>
-      <c r="G11" s="9" t="inlineStr">
-        <is>
-          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>DOUBLE_FIRE</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>app banner viewed</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>app banner viewed double-fires (gtm)</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>13 redundant payload(s) across 13 step(s); worst case 2 identical calls within 2s (e.g. "home:loaded").</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>Inflated volume; every rate computed against this event is wrong.</t>
-        </is>
-      </c>
-      <c r="G12" s="9" t="inlineStr">
-        <is>
-          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -9757,32 +9745,32 @@
       </c>
       <c r="B13" s="9" t="inlineStr">
         <is>
-          <t>DOUBLE_FIRE</t>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Ad Blocker</t>
+          <t>App Banner Viewed</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">
         <is>
-          <t>Ad Blocker double-fires (gtm)</t>
+          <t>App Banner Viewed reaches ga4 but never PostHog</t>
         </is>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>2 redundant payload(s) across 2 step(s); worst case 2 identical calls within 2s (e.g. "home:loaded").</t>
+          <t>45 captures to ga4 during this run; 0 to PostHog.</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Inflated volume; every rate computed against this event is wrong.</t>
+          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
+          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
         </is>
       </c>
     </row>
@@ -9794,32 +9782,32 @@
       </c>
       <c r="B14" s="9" t="inlineStr">
         <is>
-          <t>DOUBLE_FIRE</t>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Private Mode Modal</t>
+          <t>Plus Lock</t>
         </is>
       </c>
       <c r="D14" s="12" t="inlineStr">
         <is>
-          <t>Private Mode Modal double-fires (gtm)</t>
+          <t>Plus Lock reaches ga4 but never PostHog</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>12 redundant payload(s) across 12 step(s); worst case 2 identical calls within 2s (e.g. "home:loaded").</t>
+          <t>35 captures to ga4 during this run; 0 to PostHog.</t>
         </is>
       </c>
       <c r="F14" s="9" t="inlineStr">
         <is>
-          <t>Inflated volume; every rate computed against this event is wrong.</t>
+          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
         <is>
-          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
+          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
         </is>
       </c>
     </row>
@@ -9831,32 +9819,32 @@
       </c>
       <c r="B15" s="9" t="inlineStr">
         <is>
-          <t>DOUBLE_FIRE</t>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>app banner clicked</t>
+          <t>scroll</t>
         </is>
       </c>
       <c r="D15" s="12" t="inlineStr">
         <is>
-          <t>app banner clicked double-fires (gtm)</t>
+          <t>scroll reaches ga4 but never PostHog</t>
         </is>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>1 redundant payload(s) across 1 step(s); worst case 2 identical calls within 2s (e.g. "recirc:tag").</t>
+          <t>18 captures to ga4 during this run; 0 to PostHog.</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Inflated volume; every rate computed against this event is wrong.</t>
+          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
+          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
         </is>
       </c>
     </row>
@@ -9868,32 +9856,32 @@
       </c>
       <c r="B16" s="9" t="inlineStr">
         <is>
-          <t>GTM_ONLY</t>
+          <t>COVERAGE_GAP</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>scroll_depth</t>
+          <t>Scroll Depth</t>
         </is>
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>scroll_depth reaches GTM/Meta but never PostHog</t>
+          <t>Scroll Depth reaches ga4 but never PostHog</t>
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>Confirmed live this run: fires as Custom Scroll Depth on the GTM/Meta path with 0 PostHog captures.</t>
+          <t>2 captures to ga4 during this run; 0 to PostHog.</t>
         </is>
       </c>
       <c r="F16" s="9" t="inlineStr">
         <is>
-          <t>The ad platform can optimise on this signal; product analytics cannot see it. P1 #5: fires to GTM+Meta only, PostHog gets 0. Also double-fires w/ ScrollDepth-Value-Calculator</t>
+          <t>The ad platform can optimise on this behaviour. The tool you make product decisions in cannot see it.</t>
         </is>
       </c>
       <c r="G16" s="9" t="inlineStr">
         <is>
-          <t>Emit scroll_depth to PostHog with its spec'd property groups.</t>
+          <t>Mirror the event to PostHog through the shared transform layer, or decide deliberately that it is marketing-only and record that.</t>
         </is>
       </c>
     </row>
@@ -9905,32 +9893,32 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>NOT_INSTRUMENTED</t>
+          <t>DOUBLE_FIRE</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>read_time_logged</t>
+          <t>app banner viewed</t>
         </is>
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>read_time_logged is not instrumented at all</t>
+          <t>app banner viewed double-fires (gtm)</t>
         </is>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>No production event is mapped to this spec event (status: missing).</t>
+          <t>30 redundant payload(s) across 25 step(s); worst case 4 identical calls within 2s (e.g. "home:loaded").</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Engaged-read time; Plus-content value proof</t>
+          <t>Inflated volume; every rate computed against this event is wrong.</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Instrument read_time_logged per the spec — fires when: Active read time on an article (on unload / 30s beacon).</t>
+          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -9942,32 +9930,32 @@
       </c>
       <c r="B18" s="9" t="inlineStr">
         <is>
-          <t>NOT_INSTRUMENTED</t>
+          <t>DOUBLE_FIRE</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>freewall_cta_clicked</t>
+          <t>Private Mode Modal</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>freewall_cta_clicked is not instrumented at all</t>
+          <t>Private Mode Modal double-fires (gtm)</t>
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr">
         <is>
-          <t>No production event is mapped to this spec event (status: missing).</t>
+          <t>24 redundant payload(s) across 20 step(s); worst case 4 identical calls within 2s (e.g. "home:loaded").</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
         <is>
-          <t>Freewall → auth funnel</t>
+          <t>Inflated volume; every rate computed against this event is wrong.</t>
         </is>
       </c>
       <c r="G18" s="9" t="inlineStr">
         <is>
-          <t>Instrument freewall_cta_clicked per the spec — fires when: User taps the register CTA on the freewall.</t>
+          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -9979,32 +9967,32 @@
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>NOT_INSTRUMENTED</t>
+          <t>DOUBLE_FIRE</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>nav_clicked</t>
+          <t>Custom Scroll Depth</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>nav_clicked is not instrumented at all</t>
+          <t>Custom Scroll Depth double-fires (gtm)</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>No production event is mapped to this spec event (status: missing).</t>
+          <t>1 redundant payload(s) across 1 step(s); worst case 2 identical calls within 2s (e.g. "freewall:article-4").</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>IA usage; menu heat</t>
+          <t>Inflated volume; every rate computed against this event is wrong.</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Instrument nav_clicked per the spec — fires when: Header / sub-nav / footer link tapped.</t>
+          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -10016,32 +10004,32 @@
       </c>
       <c r="B20" s="9" t="inlineStr">
         <is>
-          <t>NOT_INSTRUMENTED</t>
+          <t>DOUBLE_FIRE</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>listing_viewed</t>
+          <t>Save Story</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>listing_viewed is not instrumented at all</t>
+          <t>Save Story double-fires (gtm)</t>
         </is>
       </c>
       <c r="E20" s="9" t="inlineStr">
         <is>
-          <t>No production event is mapped to this spec event (status: partial).</t>
+          <t>1 redundant payload(s) across 1 step(s); worst case 2 identical calls within 2s (e.g. "auth:save-story").</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
         <is>
-          <t>Section reach; author &amp; topic hub usage</t>
+          <t>Inflated volume; every rate computed against this event is wrong.</t>
         </is>
       </c>
       <c r="G20" s="9" t="inlineStr">
         <is>
-          <t>Instrument listing_viewed per the spec — fires when: A listing page loads — CONSOLIDATED across page kinds.</t>
+          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -10053,32 +10041,32 @@
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>NOT_INSTRUMENTED</t>
+          <t>DOUBLE_FIRE</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>tag_clicked</t>
+          <t>scroll_depth</t>
         </is>
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>tag_clicked is not instrumented at all</t>
+          <t>scroll_depth double-fires (gtm)</t>
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>No production event is mapped to this spec event (status: missing).</t>
+          <t>318 redundant payload(s) across 305 step(s); worst case 6 identical calls within 2s (e.g. "auth:my-inc42").</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Topic-graph navigation</t>
+          <t>Inflated volume; every rate computed against this event is wrong.</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>Instrument tag_clicked per the spec — fires when: An inline tag / industry chip on an article is tapped.</t>
+          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -10090,32 +10078,32 @@
       </c>
       <c r="B22" s="9" t="inlineStr">
         <is>
-          <t>PAGE_ERROR</t>
+          <t>DOUBLE_FIRE</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>(runtime)</t>
+          <t>Page View</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>Uncaught page error: Uncaught TypeError: undefined is not iterable (cannot read property Sy</t>
+          <t>Page View double-fires (gtm)</t>
         </is>
       </c>
       <c r="E22" s="9" t="inlineStr">
         <is>
-          <t>Thrown 22× during 20 journey step(s): article-read:start, home:loaded, article:scrolled.</t>
+          <t>2 redundant payload(s) across 1 step(s); worst case 3 identical calls within 2s (e.g. "auth:my-inc42").</t>
         </is>
       </c>
       <c r="F22" s="9" t="inlineStr">
         <is>
-          <t>An uncaught error aborts the rest of its call stack — any analytics call queued after it never runs.</t>
+          <t>Inflated volume; every rate computed against this event is wrong.</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
         <is>
-          <t>Fix the error, or move analytics calls ahead of the throwing code.</t>
+          <t>Find the duplicate listener — usually an SPA re-render or a handler bound twice.</t>
         </is>
       </c>
     </row>
@@ -10127,32 +10115,32 @@
       </c>
       <c r="B23" s="9" t="inlineStr">
         <is>
-          <t>PROP_MISSING</t>
+          <t>GTM_ONLY</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>search_initiated</t>
+          <t>scroll_depth</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Search Active is missing 1 spec'd property</t>
+          <t>scroll_depth reaches GTM/Meta but never PostHog</t>
         </is>
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Missing: surface. Captured keys: Domain, Page Title, Page URL, Page Type, User Type, User State, Referring URL, Device Type, $os, $os_version, $browser, $device_type, $timezone, $timezone_offset…</t>
+          <t>Confirmed live this run: fires as Custom Scroll Depth on the GTM/Meta path with 0 PostHog captures.</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>The dimension the event exists to slice by is unavailable.</t>
+          <t>The ad platform can optimise on this signal; product analytics cannot see it. P1 #5: fires to GTM+Meta only, PostHog gets 0. Also double-fires w/ ScrollDepth-Value-Calculator</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Attach surface at the call site.</t>
+          <t>Emit scroll_depth to PostHog with its spec'd property groups.</t>
         </is>
       </c>
     </row>
@@ -10164,32 +10152,32 @@
       </c>
       <c r="B24" s="9" t="inlineStr">
         <is>
-          <t>PROP_MISSING</t>
+          <t>NEVER_IDENTIFIED</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>search_performed</t>
+          <t>(identity)</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Search Completed is missing 3 spec'd properties</t>
+          <t>The same signed-in user carries 3 different distinct_ids</t>
         </is>
       </c>
       <c r="E24" s="9" t="inlineStr">
         <is>
-          <t>Missing: query, search_scope, result_count. Captured keys: Domain, Page Title, Page URL, Page Type, User Type, User State, Referring URL, Search Query, $os, $os_version, $browser, $device_type, $timezone, $timezone_offset…</t>
+          <t>Observed: 01a02fb4-02ac…, 01a02fb8-d550…, 01a02fb9-b468… — one per browser context, with no identify() to merge them.</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
         <is>
-          <t>The dimension the event exists to slice by is unavailable.</t>
+          <t>One person is counted as several. Person-level metrics and any retention or frequency number are inflated.</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
         <is>
-          <t>Attach query, search_scope, result_count at the call site.</t>
+          <t>Identify on load so contexts converge on the Auth0 uid.</t>
         </is>
       </c>
     </row>
@@ -10201,32 +10189,32 @@
       </c>
       <c r="B25" s="9" t="inlineStr">
         <is>
-          <t>PROP_MISSING</t>
+          <t>NOT_INSTRUMENTED</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>search_result_clicked</t>
+          <t>read_time_logged</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Search Click is missing 2 spec'd properties</t>
+          <t>read_time_logged is not instrumented at all</t>
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Missing: query, position. Captured keys: Domain, Page Title, Page URL, Page Type, User Type, User State, Referring URL, Search Query, Result Count, Index, Result Type</t>
+          <t>No production event is mapped to this spec event (status: missing).</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>The dimension the event exists to slice by is unavailable.</t>
+          <t>Engaged-read time; Plus-content value proof</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Attach query, position at the call site.</t>
+          <t>Instrument read_time_logged per the spec — fires when: Active read time on an article (on unload / 30s beacon).</t>
         </is>
       </c>
     </row>
@@ -10238,407 +10226,740 @@
       </c>
       <c r="B26" s="9" t="inlineStr">
         <is>
+          <t>NOT_INSTRUMENTED</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>freewall_cta_clicked</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>freewall_cta_clicked is not instrumented at all</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>No production event is mapped to this spec event (status: missing).</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Freewall → auth funnel</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Instrument freewall_cta_clicked per the spec — fires when: User taps the register CTA on the freewall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>NOT_INSTRUMENTED</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>nav_clicked</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>nav_clicked is not instrumented at all</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>No production event is mapped to this spec event (status: missing).</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>IA usage; menu heat</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Instrument nav_clicked per the spec — fires when: Header / sub-nav / footer link tapped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B28" s="9" t="inlineStr">
+        <is>
+          <t>NOT_INSTRUMENTED</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>listing_viewed</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>listing_viewed is not instrumented at all</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>No production event is mapped to this spec event (status: partial).</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Section reach; author &amp; topic hub usage</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Instrument listing_viewed per the spec — fires when: A listing page loads — CONSOLIDATED across page kinds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>NOT_INSTRUMENTED</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>tag_clicked</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>tag_clicked is not instrumented at all</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>No production event is mapped to this spec event (status: missing).</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Topic-graph navigation</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Instrument tag_clicked per the spec — fires when: An inline tag / industry chip on an article is tapped.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="inlineStr">
+        <is>
+          <t>PAGE_ERROR</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="inlineStr">
+        <is>
+          <t>(runtime)</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Uncaught page error: Uncaught TypeError: undefined is not iterable (cannot read property Sy</t>
+        </is>
+      </c>
+      <c r="E30" s="9" t="inlineStr">
+        <is>
+          <t>Thrown 34× during 32 journey step(s): article-read:start, home:loaded, article:scrolled.</t>
+        </is>
+      </c>
+      <c r="F30" s="9" t="inlineStr">
+        <is>
+          <t>An uncaught error aborts the rest of its call stack — any analytics call queued after it never runs.</t>
+        </is>
+      </c>
+      <c r="G30" s="9" t="inlineStr">
+        <is>
+          <t>Fix the error, or move analytics calls ahead of the throwing code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
+        <is>
+          <t>PAGE_ERROR</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>(runtime)</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Uncaught page error: TypeError: Cannot read properties of undefined (reading 'map')</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Thrown 2× during 2 journey step(s): freewall:article-9, freewall:article-13.</t>
+        </is>
+      </c>
+      <c r="F31" s="9" t="inlineStr">
+        <is>
+          <t>An uncaught error aborts the rest of its call stack — any analytics call queued after it never runs.</t>
+        </is>
+      </c>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>Fix the error, or move analytics calls ahead of the throwing code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="inlineStr">
+        <is>
+          <t>PROP_MISSING</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>search_initiated</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Search Active is missing 1 spec'd property</t>
+        </is>
+      </c>
+      <c r="E32" s="9" t="inlineStr">
+        <is>
+          <t>Missing: surface. Captured keys: Domain, Page Title, Page URL, Page Type, User Type, User State, Referring URL, Device Type, $os, $os_version, $browser, $device_type, $timezone, $timezone_offset…</t>
+        </is>
+      </c>
+      <c r="F32" s="9" t="inlineStr">
+        <is>
+          <t>The dimension the event exists to slice by is unavailable.</t>
+        </is>
+      </c>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>Attach surface at the call site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="inlineStr">
+        <is>
+          <t>PROP_MISSING</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>search_performed</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Search Completed is missing 3 spec'd properties</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="inlineStr">
+        <is>
+          <t>Missing: query, search_scope, result_count. Captured keys: Domain, Page Title, Page URL, Page Type, User Type, User State, Referring URL, Search Query, $os, $os_version, $browser, $device_type, $timezone, $timezone_offset…</t>
+        </is>
+      </c>
+      <c r="F33" s="9" t="inlineStr">
+        <is>
+          <t>The dimension the event exists to slice by is unavailable.</t>
+        </is>
+      </c>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>Attach query, search_scope, result_count at the call site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="inlineStr">
+        <is>
+          <t>PROP_MISSING</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>search_result_clicked</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Search Click is missing 2 spec'd properties</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="inlineStr">
+        <is>
+          <t>Missing: query, position. Captured keys: Domain, Page Title, Page URL, Page Type, User Type, User State, Referring URL, Search Query, Result Count, Index, Result Type</t>
+        </is>
+      </c>
+      <c r="F34" s="9" t="inlineStr">
+        <is>
+          <t>The dimension the event exists to slice by is unavailable.</t>
+        </is>
+      </c>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>Attach query, position at the call site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="inlineStr">
+        <is>
+          <t>PROP_MISSING</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>story_saved</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>Save Story is missing 1 spec'd property</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>Missing: source. Captured keys: Domain, Author Name, Publishing Year, Categories, Post Tags, Post Date Day, Post Date Month, Author Type, Publishing Date, Publish Time Range, Post ID, Story Type, Primary Industry, Company Type…</t>
+        </is>
+      </c>
+      <c r="F35" s="9" t="inlineStr">
+        <is>
+          <t>The dimension the event exists to slice by is unavailable.</t>
+        </is>
+      </c>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>Attach source at the call site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B36" s="9" t="inlineStr">
+        <is>
           <t>VENDOR_ASYMMETRY</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="C36" s="8" t="inlineStr">
         <is>
           <t>Search Click</t>
         </is>
       </c>
-      <c r="D26" s="12" t="inlineStr">
+      <c r="D36" s="12" t="inlineStr">
         <is>
           <t>Search Click: PostHog gets 11 properties, ads tools get 33</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>Same user action, same moment — the ad platform receives the full bundle while product analytics receives 11.</t>
         </is>
       </c>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>The tool you make product decisions in is the one starved of context.</t>
         </is>
       </c>
-      <c r="G26" s="9" t="inlineStr">
+      <c r="G36" s="9" t="inlineStr">
         <is>
           <t>Attach the shared Super + Story bundle to the PostHog call through the same transform layer.</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="14" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C27" s="8" t="inlineStr">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>session_started</t>
         </is>
       </c>
-      <c r="D27" s="12" t="inlineStr">
+      <c r="D37" s="12" t="inlineStr">
         <is>
           <t>session_started not observed — unverified</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
+      <c r="E37" s="9" t="inlineStr">
         <is>
           <t>session_start produced no captures in "article-read". No PostHog key was supplied, so production volume could not be checked.</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G37" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="14" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="C38" s="8" t="inlineStr">
         <is>
           <t>freewall_shown</t>
         </is>
       </c>
-      <c r="D28" s="12" t="inlineStr">
+      <c r="D38" s="12" t="inlineStr">
         <is>
           <t>freewall_shown not observed — unverified</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>Freewall Lock produced no captures in "freewall". No PostHog key was supplied, so production volume could not be checked.</t>
         </is>
       </c>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G28" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="14" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C29" s="8" t="inlineStr">
+      <c r="C39" s="8" t="inlineStr">
         <is>
           <t>sign_in_prompt_shown</t>
         </is>
       </c>
-      <c r="D29" s="12" t="inlineStr">
+      <c r="D39" s="12" t="inlineStr">
         <is>
           <t>sign_in_prompt_shown not observed — unverified</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
+      <c r="E39" s="9" t="inlineStr">
         <is>
           <t>Login Modal produced no captures in "freewall". No PostHog key was supplied, so production volume could not be checked.</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G39" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="14" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B30" s="9" t="inlineStr">
+      <c r="B40" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="C40" s="8" t="inlineStr">
         <is>
           <t>newsletter_subscribed</t>
         </is>
       </c>
-      <c r="D30" s="12" t="inlineStr">
+      <c r="D40" s="12" t="inlineStr">
         <is>
           <t>newsletter_subscribed not observed — unverified</t>
         </is>
       </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="E40" s="9" t="inlineStr">
         <is>
           <t>Newsletter Subscribed produced no captures in "newsletter". No PostHog key was supplied, so production volume could not be checked.</t>
         </is>
       </c>
-      <c r="F30" s="9" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G30" s="9" t="inlineStr">
+      <c r="G40" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="14" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B41" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C31" s="8" t="inlineStr">
+      <c r="C41" s="8" t="inlineStr">
         <is>
           <t>recommended_clicked</t>
         </is>
       </c>
-      <c r="D31" s="12" t="inlineStr">
+      <c r="D41" s="12" t="inlineStr">
         <is>
           <t>recommended_clicked not observed — unverified</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr">
+      <c r="E41" s="9" t="inlineStr">
         <is>
           <t>Recommendation Click produced no captures in "recirculation". No PostHog key was supplied, so production volume could not be checked.</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G41" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B32" s="9" t="inlineStr">
+      <c r="B42" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
-        <is>
-          <t>sign_in_completed</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
-        <is>
-          <t>sign_in_completed not observed — unverified</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>Login produced no captures in "logged-in". No PostHog key was supplied, so production volume could not be checked.</t>
-        </is>
-      </c>
-      <c r="F32" s="9" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
+        <is>
+          <t>entity_followed</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>entity_followed not observed — unverified</t>
+        </is>
+      </c>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Follow produced no captures in "logged-in". No PostHog key was supplied, so production volume could not be checked.</t>
+        </is>
+      </c>
+      <c r="F42" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G32" s="9" t="inlineStr">
+      <c r="G42" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="14" t="inlineStr">
+    <row r="43">
+      <c r="A43" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B43" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C33" s="8" t="inlineStr">
-        <is>
-          <t>story_saved</t>
-        </is>
-      </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>story_saved not observed — unverified</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="inlineStr">
-        <is>
-          <t>Save Story produced no captures in "logged-in". No PostHog key was supplied, so production volume could not be checked.</t>
-        </is>
-      </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>feed_viewed</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>feed_viewed not observed — unverified</t>
+        </is>
+      </c>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>My Inc42 produced no captures in "logged-in". No PostHog key was supplied, so production volume could not be checked.</t>
+        </is>
+      </c>
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G43" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="14" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B34" s="9" t="inlineStr">
+      <c r="B44" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
-        <is>
-          <t>entity_followed</t>
-        </is>
-      </c>
-      <c r="D34" s="12" t="inlineStr">
-        <is>
-          <t>entity_followed not observed — unverified</t>
-        </is>
-      </c>
-      <c r="E34" s="9" t="inlineStr">
-        <is>
-          <t>Follow produced no captures in "logged-in". No PostHog key was supplied, so production volume could not be checked.</t>
-        </is>
-      </c>
-      <c r="F34" s="9" t="inlineStr">
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t>story_shared</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>story_shared not observed — unverified</t>
+        </is>
+      </c>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Share produced no captures in "share". No PostHog key was supplied, so production volume could not be checked.</t>
+        </is>
+      </c>
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G34" s="9" t="inlineStr">
+      <c r="G44" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="14" t="inlineStr">
+    <row r="45">
+      <c r="A45" s="14" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B45" s="9" t="inlineStr">
         <is>
           <t>UNVERIFIED</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t>signed_out</t>
         </is>
       </c>
-      <c r="D35" s="12" t="inlineStr">
+      <c r="D45" s="12" t="inlineStr">
         <is>
           <t>signed_out not observed — unverified</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
-        <is>
-          <t>Logout produced no captures in "logged-in". No PostHog key was supplied, so production volume could not be checked.</t>
-        </is>
-      </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Logout produced no captures in "logout". No PostHog key was supplied, so production volume could not be checked.</t>
+        </is>
+      </c>
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G45" s="9" t="inlineStr">
         <is>
           <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="14" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="B36" s="9" t="inlineStr">
-        <is>
-          <t>UNVERIFIED</t>
-        </is>
-      </c>
-      <c r="C36" s="8" t="inlineStr">
-        <is>
-          <t>story_shared</t>
-        </is>
-      </c>
-      <c r="D36" s="12" t="inlineStr">
-        <is>
-          <t>story_shared not observed — unverified</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="inlineStr">
-        <is>
-          <t>Share produced no captures in "share". No PostHog key was supplied, so production volume could not be checked.</t>
-        </is>
-      </c>
-      <c r="F36" s="9" t="inlineStr">
-        <is>
-          <t>Cannot distinguish a broken event from a journey that never reached the trigger.</t>
-        </is>
-      </c>
-      <c r="G36" s="9" t="inlineStr">
-        <is>
-          <t>Set POSTHOG_API_KEY and re-run to resolve this either way.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:G36"/>
+  <autoFilter ref="A4:G45"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -10653,7 +10974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -10676,7 +10997,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Captured across 8 articles, run 2026-08-23 17:26. This is what 'not triggering properly' looks like in detail.</t>
+          <t>Captured across 8 articles, run 2026-08-23 17:39. This is what 'not triggering properly' looks like in detail.</t>
         </is>
       </c>
     </row>
@@ -10725,12 +11046,12 @@
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>GTM built-in scroll trigger</t>
+          <t>—</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>gtm.scrollDepth</t>
+          <t>scroll_depth</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
@@ -10740,21 +11061,21 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>25 / 50 / 75 / 90 / 100</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>gtm.scrollThreshold</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>number (25)</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G5" s="10" t="n">
-        <v>69</v>
+        <v>724</v>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
@@ -10765,80 +11086,80 @@
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
         <is>
-          <t>GA4 enhanced measurement</t>
+          <t>GTM built-in scroll trigger</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>scroll</t>
+          <t>gtm.scrollDepth</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>ga4</t>
+          <t>gtm</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>25 / 50 / 75 / 90 / 100</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>percent_scrolled</t>
+          <t>gtm.scrollThreshold</t>
         </is>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>string ("90")</t>
+          <t>number (25)</t>
         </is>
       </c>
       <c r="G6" s="10" t="n">
-        <v>16</v>
+        <v>132</v>
       </c>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>on the wire</t>
+          <t>dataLayer only</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Custom GTM tag</t>
+          <t>GA4 enhanced measurement</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Custom Scroll Depth</t>
+          <t>scroll</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>gtm</t>
+          <t>ga4</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
-          <t>Scroll_Percentage</t>
+          <t>percent_scrolled</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>string ("25%")</t>
+          <t>string ("90")</t>
         </is>
       </c>
       <c r="G7" s="10" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>dataLayer only</t>
+          <t>on the wire</t>
         </is>
       </c>
     </row>
@@ -10855,7 +11176,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>meta</t>
+          <t>gtm</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
@@ -10874,7 +11195,7 @@
         </is>
       </c>
       <c r="G8" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H8" s="9" t="inlineStr">
         <is>
@@ -10885,17 +11206,17 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Custom GTM tag → GA4</t>
+          <t>Custom GTM tag</t>
         </is>
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Scroll Depth</t>
+          <t>Custom Scroll Depth</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>ga4</t>
+          <t>meta</t>
         </is>
       </c>
       <c r="D9" s="8" t="inlineStr">
@@ -10914,152 +11235,192 @@
         </is>
       </c>
       <c r="G9" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>on the wire</t>
+          <t>dataLayer only</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
         <is>
+          <t>Custom GTM tag → GA4</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Scroll Depth</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>ga4</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>Scroll_Percentage</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>string ("25%")</t>
+        </is>
+      </c>
+      <c r="G10" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>on the wire</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
           <t>PostHog</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="8" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>posthog</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F10" s="9" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G10" s="10" t="n">
+      <c r="G11" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="11" t="inlineStr">
+      <c r="H11" s="11" t="inlineStr">
         <is>
           <t>NEVER FIRES</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>WHAT'S WRONG</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="30" customHeight="1">
-      <c r="A13" s="17" t="inlineStr">
-        <is>
-          <t>PostHog receives nothing</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Zero scroll events across 8 articles. The core editorial engagement signal is absent from the tool product decisions are made in.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>Three parallel implementations</t>
+          <t>PostHog receives nothing</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>GTM's built-in trigger, a 'Custom Scroll Depth' tag, and a 'ScrollDepth-Value-Calculator' tag all fire on the same scroll.</t>
+          <t>Zero scroll events across 8 articles. The core editorial engagement signal is absent from the tool product decisions are made in.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>Thresholds don't match the plan</t>
+          <t>Three parallel implementations</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Plan says 25/50/75/100. Production fires at 25/50/75/90/100 — the 90 threshold is undocumented and the most frequent of all.</t>
+          <t>GTM's built-in trigger, a 'Custom Scroll Depth' tag, and a 'ScrollDepth-Value-Calculator' tag all fire on the same scroll.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>GA4 gets two different events</t>
+          <t>Thresholds don't match the plan</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>'scroll' (enhanced measurement, only ever at 90) and 'Scroll Depth' (custom, at 25/50). Two names for one action; neither alone is the full curve.</t>
+          <t>Plan says 25/50/75/100. Production fires at 25/50/75/90/100 — the 90 threshold is undocumented and the most frequent of all.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="17" t="inlineStr">
         <is>
-          <t>Three formats for one number</t>
+          <t>GA4 gets two different events</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>gtm.scrollThreshold = 25 (number) · Scroll_Percentage = "25%" (string with %) · percent_scrolled = "90" (string, no %). No consumer can join these.</t>
+          <t>'scroll' (enhanced measurement, only ever at 90) and 'Scroll Depth' (custom, at 25/50). Two names for one action; neither alone is the full curve.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>Custom tag is unreliable</t>
+          <t>Three formats for one number</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>'Custom Scroll Depth' fired on only 4 of 8 articles and never above 50%. The deep-read signal — 75% and 100% — is not captured anywhere except GTM's internal dataLayer.</t>
+          <t>gtm.scrollThreshold = 25 (number) · Scroll_Percentage = "25%" (string with %) · percent_scrolled = "90" (string, no %). No consumer can join these.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="17" t="inlineStr">
         <is>
+          <t>Custom tag is unreliable</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>'Custom Scroll Depth' fired on only 4 of 8 articles and never above 50%. The deep-read signal — 75% and 100% — is not captured anywhere except GTM's internal dataLayer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
           <t>Genuine double-fire</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr">
         <is>
           <t>'Custom Scroll Depth' and 'ScrollDepth-Value-Calculator' each emit duplicate payloads within 2s at the same threshold.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="46" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="22" ht="46" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
         <is>
           <t>FIX</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Emit one canonical scroll_depth event to PostHog at 25/50/75/100 carrying the Super + Story bundle and depth_percent as an integer. Retire the two custom GTM tags; keep the Meta value as a property on the one event, not a second event. Decide whether 90 stays (GA4 enhanced measurement) and document it if so.</t>
         </is>
@@ -11067,16 +11428,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B22:H22"/>
     <mergeCell ref="B14:H14"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B13:H13"/>
-    <mergeCell ref="B21:H21"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B15:H15"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B19:H19"/>
+    <mergeCell ref="B20:H20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>